<commit_message>
Verify replication-package kit and link it from its niche
Re-ran the checker (34 findings on the original sample, none on the
fixed package) and the reproduction run (4 of 4 outputs identical).
README now says to install the package's own dependencies first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/board-minutes/samples/wrenfield-commons-2026-09-16-motions.xlsx
+++ b/kits/board-minutes/samples/wrenfield-commons-2026-09-16-motions.xlsx
@@ -130,7 +130,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -138,11 +138,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
@@ -626,7 +626,7 @@
           <t>Motion 1</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -648,7 +648,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>voice vote</t>
+          <t>Voice vote</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
@@ -676,7 +676,7 @@
           <t>Motion 2</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -691,19 +691,19 @@
           <t>Marcus Bell</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>[UNCLEAR: Raymond Castillo or Grace Lindqvist]</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>voice vote</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
+          <t>Voice vote</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Carried</t>
@@ -726,7 +726,7 @@
           <t>Motion 3</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>8a</t>
         </is>
@@ -748,7 +748,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>voice vote</t>
+          <t>Voice vote</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
@@ -776,7 +776,7 @@
           <t>Motion 4</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>9a</t>
         </is>
@@ -798,16 +798,16 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>roll call vote</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="n">
+          <t>Roll call vote</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="9" t="n"/>
+      <c r="I8" s="8" t="n"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Carried</t>
@@ -830,7 +830,7 @@
           <t>Motion 5</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>9b</t>
         </is>
@@ -852,7 +852,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>voice vote</t>
+          <t>Voice vote</t>
         </is>
       </c>
       <c r="G9" s="5" t="n">
@@ -880,7 +880,7 @@
           <t>Motion 6</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>9c</t>
         </is>
@@ -898,16 +898,16 @@
       <c r="E10" s="7" t="inlineStr"/>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>voice vote</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="n">
+          <t>Voice vote</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="H10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -932,7 +932,7 @@
           <t>Motion 7</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -954,7 +954,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>voice vote</t>
+          <t>Voice vote</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
@@ -986,7 +986,7 @@
           <t>Motion 8</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -1008,12 +1008,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>voice vote</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
+          <t>Voice vote</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
       <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Carried</t>
@@ -1111,7 +1111,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1127,7 +1127,7 @@
       <c r="D5" s="10" t="n">
         <v>46316</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1144,7 +1144,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1152,7 +1152,7 @@
           <t>Look into adding a pet-waste bag station near the playground, including the cost.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>[UNCLEAR]</t>
         </is>
@@ -1160,7 +1160,7 @@
       <c r="D6" s="11" t="n">
         <v>46316</v>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1177,7 +1177,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1195,7 +1195,7 @@
           <t>Budget workshop</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1212,7 +1212,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1230,7 +1230,7 @@
           <t>Until repaired</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -1247,7 +1247,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1263,7 +1263,7 @@
       <c r="D9" s="10" t="n">
         <v>46316</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>8a</t>
         </is>
@@ -1280,7 +1280,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1296,7 +1296,7 @@
       <c r="D10" s="11" t="n">
         <v>46283</v>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>9a</t>
         </is>
@@ -1313,7 +1313,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1329,7 +1329,7 @@
       <c r="D11" s="10" t="n">
         <v>46295</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>9b</t>
         </is>
@@ -1346,7 +1346,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1362,7 +1362,7 @@
       <c r="D12" s="11" t="n">
         <v>46283</v>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>9c</t>
         </is>
@@ -1379,7 +1379,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1395,7 +1395,7 @@
       <c r="D13" s="10" t="n">
         <v>46282</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -1489,7 +1489,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1510,7 +1510,7 @@
       <c r="E5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1531,7 +1531,7 @@
       <c r="E6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1552,7 +1552,7 @@
       <c r="E7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>[UNCLEAR] markers</t>
         </is>

</xml_diff>